<commit_message>
Build v5.6: Added Modern Admin GUI, Scrollable Engineer Panel, and QR Printing Studio
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,7 +469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>test1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -484,33 +484,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>test2</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>500</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -524,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,55 +541,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Amit Patil</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-04-16 12:51:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Suresh Kumar</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-04-16 13:00:29</t>
+          <t>2026-04-16 15:16:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build v5.7: Fixed CP/SP/Stock column mapping and improved Dashboard Analytics
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +485,32 @@
       </c>
       <c r="F2" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>filter</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>250</v>
+      </c>
+      <c r="D3" t="n">
+        <v>900</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OG</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New Feature TCR Tracking is Implement
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service_Billing" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,12 +32,24 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -57,11 +70,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,7 +502,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -776,7 +793,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -820,7 +836,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -864,7 +879,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -908,7 +922,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>IN</t>
@@ -927,7 +940,6 @@
           <t>2026-04-17 11:02:12</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>2026-04-17 11:02:12</t>
@@ -948,7 +960,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -962,7 +973,6 @@
       <c r="G6" t="n">
         <v>4000</v>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>2026-04-17 11:16:50</t>
@@ -988,29 +998,32 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>vishal</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-04-17 11:02:12</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-04-18 17:11:39</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-17 11:02:12</t>
+          <t>2026-04-18 17:11:39</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1041,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1047,7 +1059,6 @@
           <t>2026-04-17 11:02:12</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>2026-04-17 11:02:12</t>
@@ -1068,7 +1079,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1087,7 +1097,6 @@
           <t>2026-04-17 11:02:12</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>2026-04-17 11:02:12</t>
@@ -1108,7 +1117,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1122,7 +1130,6 @@
       <c r="G10" t="n">
         <v>4000</v>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>2026-04-17 11:17:14</t>
@@ -1148,7 +1155,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1167,7 +1173,6 @@
           <t>2026-04-17 11:02:12</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>2026-04-17 11:02:12</t>
@@ -1188,7 +1193,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1202,7 +1206,6 @@
       <c r="G12" t="n">
         <v>1000</v>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>2026-04-17 11:29:07</t>
@@ -1228,7 +1231,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1242,7 +1244,6 @@
       <c r="G13" t="n">
         <v>1000</v>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>2026-04-17 11:30:54</t>
@@ -1268,7 +1269,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1287,7 +1287,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1308,7 +1307,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1322,7 +1320,6 @@
       <c r="G15" t="n">
         <v>1000</v>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>2026-04-17 11:30:29</t>
@@ -1348,7 +1345,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1362,7 +1358,6 @@
       <c r="G16" t="n">
         <v>1000</v>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>2026-04-17 11:31:13</t>
@@ -1388,7 +1383,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1407,7 +1401,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1428,7 +1421,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1447,7 +1439,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1468,7 +1459,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1487,7 +1477,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1508,7 +1497,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1527,7 +1515,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1548,7 +1535,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1567,7 +1553,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1588,7 +1573,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1607,7 +1591,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1628,7 +1611,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1647,7 +1629,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1668,7 +1649,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1687,7 +1667,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1708,7 +1687,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1727,7 +1705,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1748,7 +1725,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1767,7 +1743,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1788,7 +1763,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1807,7 +1781,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1828,7 +1801,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1847,7 +1819,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1868,7 +1839,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>OUT</t>
@@ -1882,7 +1852,6 @@
       <c r="G29" t="n">
         <v>1000</v>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>2026-04-17 11:08:57</t>
@@ -1908,7 +1877,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1927,7 +1895,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -1948,7 +1915,6 @@
           <t>Company</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>IN</t>
@@ -1967,7 +1933,6 @@
           <t>2026-04-17 11:07:54</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>2026-04-17 11:07:54</t>
@@ -2011,7 +1976,6 @@
           <t>2026-04-17 11:28:54</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>2026-04-17 11:28:54</t>
@@ -2055,7 +2019,6 @@
           <t>2026-04-17 11:29:02</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>2026-04-17 11:29:02</t>
@@ -2094,7 +2057,6 @@
       <c r="G34" t="n">
         <v>6000</v>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>2026-04-17 11:34:48</t>
@@ -2143,7 +2105,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2187,7 +2148,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2231,7 +2191,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2275,7 +2234,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2319,7 +2277,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2363,7 +2320,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2407,7 +2363,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2451,7 +2406,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2495,7 +2449,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2539,7 +2492,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2583,7 +2535,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2627,7 +2578,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2671,7 +2621,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2715,7 +2664,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2759,7 +2707,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2803,7 +2750,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2847,7 +2793,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2891,7 +2836,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2935,7 +2879,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -2979,7 +2922,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3023,7 +2965,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3067,7 +3008,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3111,7 +3051,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3155,7 +3094,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3199,7 +3137,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3243,7 +3180,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3287,7 +3223,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3331,7 +3266,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3375,7 +3309,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3419,7 +3352,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3463,7 +3395,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3507,7 +3438,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3551,7 +3481,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3595,7 +3524,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3639,7 +3567,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3683,7 +3610,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3727,7 +3653,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3771,7 +3696,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3815,7 +3739,6 @@
           <t>2026-04-17 11:33:16</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>2026-04-17 11:33:16</t>
@@ -3854,7 +3777,6 @@
       <c r="G74" t="n">
         <v>300</v>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>2026-04-17 11:54:08</t>
@@ -3903,7 +3825,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -3947,7 +3868,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -3991,7 +3911,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4035,7 +3954,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4079,7 +3997,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4123,7 +4040,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4167,7 +4083,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4211,7 +4126,6 @@
           <t>2026-04-17 11:43:33</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>2026-04-17 11:43:33</t>
@@ -4250,7 +4164,6 @@
       <c r="G83" t="n">
         <v>400</v>
       </c>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>2026-04-17 11:52:49</t>
@@ -4299,7 +4212,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4343,7 +4255,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4382,7 +4293,6 @@
       <c r="G86" t="n">
         <v>400</v>
       </c>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>2026-04-17 11:52:36</t>
@@ -4431,7 +4341,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4475,7 +4384,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4514,7 +4422,6 @@
       <c r="G89" t="n">
         <v>400</v>
       </c>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>2026-04-17 11:52:07</t>
@@ -4563,7 +4470,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4607,7 +4513,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4651,7 +4556,6 @@
           <t>2026-04-17 11:51:08</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
           <t>2026-04-17 11:51:08</t>
@@ -4695,7 +4599,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4739,7 +4642,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4783,7 +4685,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4827,7 +4728,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4871,7 +4771,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4915,7 +4814,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -4959,7 +4857,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5003,7 +4900,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5047,7 +4943,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5091,7 +4986,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5135,7 +5029,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5179,7 +5072,6 @@
           <t>2026-04-17 12:13:30</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>2026-04-17 12:13:30</t>
@@ -5223,7 +5115,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5310,7 +5201,6 @@
       <c r="G107" t="n">
         <v>3500</v>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>2026-04-17 12:19:55</t>
@@ -5359,7 +5249,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5403,7 +5292,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5447,7 +5335,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5491,7 +5378,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5535,7 +5421,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5579,7 +5464,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5623,7 +5507,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5667,7 +5550,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5711,7 +5593,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5755,7 +5636,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5799,7 +5679,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5843,7 +5722,6 @@
           <t>2026-04-17 12:18:53</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>2026-04-17 12:18:53</t>
@@ -5897,8 +5775,6 @@
           <t>Yogesh Bhosale</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>True</t>
@@ -5916,8 +5792,6 @@
           <t>Sidram Battul</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>True</t>
@@ -5935,8 +5809,6 @@
           <t>Sham Kachi</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>True</t>
@@ -5954,8 +5826,6 @@
           <t>sameer shaikh</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>True</t>
@@ -5973,8 +5843,6 @@
           <t>Rajesh chavan</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>True</t>
@@ -5992,8 +5860,6 @@
           <t>Sahil Dighe</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>True</t>
@@ -6011,8 +5877,6 @@
           <t>Gajanan gawande</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>True</t>
@@ -6030,8 +5894,6 @@
           <t>Kiran misal</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>True</t>
@@ -6049,8 +5911,6 @@
           <t>kishor panchal</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>True</t>
@@ -6068,8 +5928,6 @@
           <t>Raju Yadav</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>True</t>
@@ -6087,8 +5945,6 @@
           <t>Lalemashak kunnure</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>True</t>
@@ -6106,8 +5962,6 @@
           <t>Faruk Shaikh</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>True</t>
@@ -6125,8 +5979,6 @@
           <t>Ashraf Momin</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>True</t>
@@ -6144,8 +5996,6 @@
           <t>Abhitabh Gupta</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>True</t>
@@ -6163,8 +6013,6 @@
           <t>Prahalad Yadav</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>True</t>
@@ -6182,8 +6030,6 @@
           <t>Abdul Rehman</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>True</t>
@@ -6201,8 +6047,6 @@
           <t>Ishwar Panchal</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>True</t>
@@ -6220,8 +6064,6 @@
           <t>Nagendra Yadav</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>True</t>
@@ -6239,8 +6081,6 @@
           <t>Pramod Valekar</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>True</t>
@@ -6258,8 +6098,6 @@
           <t>Rahim Dindore</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>True</t>
@@ -6295,6 +6133,236 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>2026-04-17 12:48:07</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Row_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Sr_No</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Engineer_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Job_Card_Invoice_No</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Outward_Date</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>TCR_No</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>TCR_Date</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Warranty_Warranty_No</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Bill_Amount</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Incentive</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Ticket_Closed_On_Date</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Part_Name_Part_No</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Material_Description</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>HSN_Code</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>MRP_Product_Price</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>CGST</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>SGST</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Article_No</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Part_Sr_No</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Money_Received</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>Created_At</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>Updated_At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>3363e3a3-b674-4ef0-8644-b1848f4d485a</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>vishal</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18 17:11:39</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>TCR-1nan</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>xsy</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Service work on local purchase - xsy</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr"/>
+      <c r="V2" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="X2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18 17:11:39</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18 17:12:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update features with Search bars
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -47,14 +51,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -86,6 +90,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,34 +463,42 @@
   </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Article_No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Part_Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Stock_Level</t>
         </is>
@@ -525,54 +543,66 @@
   </sheetPr>
   <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Article_No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Sr_No</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Purchase_Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Tax_Invoice_No</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Charges</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>In_Date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Out_Date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1469,41 +1499,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Engineer_Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>BP_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>PPRR_ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Created_At</t>
         </is>
@@ -1877,12 +1916,39 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>shubham</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>wf</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:16</t>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-04-21 17:05:44</t>
         </is>
       </c>
     </row>
@@ -1899,129 +1965,156 @@
   </sheetPr>
   <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Row_ID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Engineer_Name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Job_Card_Invoice_No</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Outward_Date</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>TCR_No</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>TCR_Date</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Warranty_Warranty_No</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Bill_Amount</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Incentive</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Ticket_Closed_On_Date</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Part_Name_Part_No</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Material_Description</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>HSN_Code</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>MRP_Product_Price</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>CGST</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>SGST</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>Article_No</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>Part_Sr_No</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Money_Received</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>Created_At</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>Updated_At</t>
         </is>
@@ -2088,7 +2181,7 @@
       <c r="R2" s="3" t="inlineStr"/>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr"/>
@@ -2099,257 +2192,257 @@
         <v>1</v>
       </c>
       <c r="W2" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:36</t>
+        </is>
+      </c>
+      <c r="Y2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21 17:07:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>42fdc5e7-d5ae-468f-b960-81f65bd1f3d9</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>vishal</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>sdfg</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:41</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>xz</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Service work on 🏢 company purchase - xz</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr"/>
+      <c r="U3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="W3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:41</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21 17:07:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>40918705-5523-4efa-9d8b-2e7c8b561d0b</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>vishal</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>sdfg</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:45</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>TCR-3nan</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>20-Apr-2026</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>xz</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Service work on 🏢 company purchase - xz</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:36</t>
-        </is>
-      </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-21 11:52:52</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>42fdc5e7-d5ae-468f-b960-81f65bd1f3d9</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:45</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:16:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>ef2a0047-8c8e-4c16-abb8-2b8e2fe68cb6</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>vishal</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>sdfg</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:41</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr"/>
-      <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" s="4" t="inlineStr"/>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:15:49</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>TCR-4nan</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>20-Apr-2026</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>xz</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Service work on 🏢 company purchase - xz</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr"/>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="n">
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr"/>
+      <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr"/>
+      <c r="U5" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="V3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W3" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="X3" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:41</t>
-        </is>
-      </c>
-      <c r="Y3" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:41</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>40918705-5523-4efa-9d8b-2e7c8b561d0b</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>vishal</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>sdfg</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:45</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>TCR-3nan</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>20-Apr-2026</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>xz</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Service work on 🏢 company purchase - xz</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr"/>
-      <c r="U4" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="V4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="W4" s="3" t="b">
+      <c r="V5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="W5" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="X4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:45</t>
-        </is>
-      </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:16:35</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>ef2a0047-8c8e-4c16-abb8-2b8e2fe68cb6</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>vishal</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>sdfg</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>2026-04-20 15:15:49</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>TCR-4nan</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>20-Apr-2026</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>xz</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Service work on 🏢 company purchase - xz</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr"/>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr"/>
-      <c r="R5" s="3" t="inlineStr"/>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr"/>
-      <c r="U5" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="V5" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="W5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X5" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:15:49</t>
-        </is>
-      </c>
-      <c r="Y5" s="3" t="inlineStr">
+      <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>2026-04-20 15:16:20</t>
         </is>

</xml_diff>

<commit_message>
Optimize UI and exclude build artifacts
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3265,6 +3265,92 @@
       <c r="J60" t="inlineStr">
         <is>
           <t>2026-04-22 17:05:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>26</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>vss103</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:39:35</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:39:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>27</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>vss103</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:39:35</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:39:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize UI and exclude build artifacts 2
</commit_message>
<xml_diff>
--- a/resQ_Enterprise_Inventory.xlsx
+++ b/resQ_Enterprise_Inventory.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +588,32 @@
       </c>
       <c r="F5" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>400</v>
+      </c>
+      <c r="D6" t="n">
+        <v>800</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OG</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -601,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3351,6 +3377,441 @@
       <c r="J62" t="inlineStr">
         <is>
           <t>2026-04-23 11:39:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Sidram Battul</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>800</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:46:20</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:46:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>6</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>7</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>8</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>9</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>10</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>🏢 Company</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:45:10</t>
         </is>
       </c>
     </row>
@@ -3756,7 +4217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:Y17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4616,75 +5077,87 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>78814050-1a48-4e06-91ae-f2b9530daa55</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Rahim Dindore</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>vss104</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>2026-04-22 17:06:07</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>TCR-nan</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>29-Apr-2026</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Service work on 🏪 local purchase - panel</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr"/>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr"/>
-      <c r="Q11" s="3" t="inlineStr"/>
-      <c r="R11" s="3" t="inlineStr"/>
-      <c r="S11" s="3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="T11" s="3" t="inlineStr"/>
-      <c r="U11" s="3" t="n">
+      <c r="N11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
+      <c r="Q11" s="4" t="inlineStr"/>
+      <c r="R11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr"/>
+      <c r="U11" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="V11" s="3" t="n">
+      <c r="V11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="W11" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="X11" s="3" t="inlineStr">
+      <c r="W11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
         <is>
           <t>2026-04-22 17:06:07</t>
         </is>
       </c>
-      <c r="Y11" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-22 17:06:07</t>
+      <c r="Y11" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:31:04</t>
         </is>
       </c>
     </row>
@@ -5069,6 +5542,95 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>90c41c44-8837-464a-bcf9-6c1317485127</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Sidram Battul</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>vss108</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:46:20</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>TCR-6326</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>29-Apr-2026</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Service work on 🏢 company purchase - abc</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr"/>
+      <c r="U17" s="4" t="n">
+        <v>401</v>
+      </c>
+      <c r="V17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:46:20</t>
+        </is>
+      </c>
+      <c r="Y17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:47:44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>